<commit_message>
bổ sung tài liệu
</commit_message>
<xml_diff>
--- a/Tài Liệu/SCI_SE_9.ProjectTestReport.xlsx
+++ b/Tài Liệu/SCI_SE_9.ProjectTestReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOI\Desktop\KLTN (1)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF396F1-4911-4123-A8BD-08B07BE8B3CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80CE0BF-B949-4147-942F-4DFF5FC8C8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestReportSprint1" sheetId="1" r:id="rId1"/>
@@ -322,7 +322,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -671,7 +671,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -719,7 +719,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -788,6 +788,9 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -809,18 +812,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -829,9 +832,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1149,82 +1149,82 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="44.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.25" style="1" customWidth="1"/>
+    <col min="2" max="2" width="44.25" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.21875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="16.25" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.25" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.75" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-    </row>
-    <row r="3" spans="1:7" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+    </row>
+    <row r="3" spans="1:7" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="54"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="55"/>
+      <c r="C4" s="56"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
     </row>
-    <row r="5" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="57"/>
+      <c r="C5" s="58"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
     </row>
-    <row r="6" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="56" t="s">
+    <row r="6" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="57" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>573</v>
+        <v>528</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
     </row>
-    <row r="7" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56"/>
+    <row r="7" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="57"/>
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
@@ -1236,21 +1236,21 @@
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
     </row>
-    <row r="8" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56"/>
+    <row r="8" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="57"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="8">
-        <v>573</v>
+        <v>528</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
     </row>
-    <row r="9" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="56" t="s">
+    <row r="9" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="57" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -1264,8 +1264,8 @@
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="56"/>
+    <row r="10" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="57"/>
       <c r="B10" s="3" t="s">
         <v>15</v>
       </c>
@@ -1277,8 +1277,8 @@
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
     </row>
-    <row r="11" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="56"/>
+    <row r="11" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="57"/>
       <c r="B11" s="3" t="s">
         <v>16</v>
       </c>
@@ -1290,8 +1290,8 @@
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
     </row>
-    <row r="12" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="56"/>
+    <row r="12" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="57"/>
       <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
@@ -1303,20 +1303,20 @@
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
     </row>
-    <row r="13" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="58" t="s">
+    <row r="13" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="58"/>
+      <c r="B13" s="59"/>
       <c r="C13" s="18">
-        <v>573</v>
+        <v>528</v>
       </c>
       <c r="D13" s="23"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="20"/>
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
@@ -1325,7 +1325,7 @@
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
     </row>
-    <row r="15" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>0</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="30" t="s">
         <v>29</v>
       </c>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="G16" s="35"/>
     </row>
-    <row r="17" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
         <v>28</v>
       </c>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="G17" s="35"/>
     </row>
-    <row r="18" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>43</v>
       </c>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="G18" s="35"/>
     </row>
-    <row r="19" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="32" t="s">
         <v>44</v>
       </c>
@@ -1433,7 +1433,7 @@
       <c r="G19" s="35"/>
       <c r="H19" s="29"/>
     </row>
-    <row r="20" spans="1:9" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
         <v>45</v>
       </c>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="G20" s="36"/>
     </row>
-    <row r="21" spans="1:9" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="32" t="s">
         <v>46</v>
       </c>
@@ -1477,7 +1477,7 @@
       <c r="H21" s="29"/>
       <c r="I21" s="29"/>
     </row>
-    <row r="22" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
         <v>34</v>
       </c>
@@ -1500,7 +1500,7 @@
       <c r="H22" s="29"/>
       <c r="I22" s="29"/>
     </row>
-    <row r="23" spans="1:9" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="32" t="s">
         <v>47</v>
       </c>
@@ -1523,7 +1523,7 @@
       <c r="H23" s="29"/>
       <c r="I23" s="29"/>
     </row>
-    <row r="24" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32" t="s">
         <v>48</v>
       </c>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="G24" s="35"/>
     </row>
-    <row r="25" spans="1:9" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>19</v>
       </c>
@@ -1563,8 +1563,8 @@
       <c r="F25" s="37"/>
       <c r="G25" s="38"/>
     </row>
-    <row r="26" spans="1:9" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="56" t="s">
+    <row r="26" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="57" t="s">
         <v>25</v>
       </c>
       <c r="B26" s="12" t="s">
@@ -1573,17 +1573,17 @@
       <c r="C26" s="28">
         <v>2</v>
       </c>
-      <c r="D26" s="66" t="s">
+      <c r="D26" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="66" t="s">
+      <c r="E26" s="52" t="s">
         <v>56</v>
       </c>
       <c r="F26" s="28"/>
       <c r="G26" s="28"/>
     </row>
-    <row r="27" spans="1:9" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="56"/>
+    <row r="27" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="57"/>
       <c r="B27" s="12" t="s">
         <v>23</v>
       </c>
@@ -1599,15 +1599,15 @@
       <c r="F27" s="28"/>
       <c r="G27" s="28"/>
     </row>
-    <row r="28" spans="1:9" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="56"/>
+    <row r="28" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="57"/>
       <c r="B28" s="12" t="s">
         <v>24</v>
       </c>
       <c r="C28" s="28">
         <v>1</v>
       </c>
-      <c r="D28" s="66" t="s">
+      <c r="D28" s="52" t="s">
         <v>56</v>
       </c>
       <c r="E28" s="35" t="s">
@@ -1627,60 +1627,60 @@
     <mergeCell ref="A9:A12"/>
     <mergeCell ref="A13:B13"/>
   </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.74803149606299213" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:G29"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="47.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.21875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="34.75" style="1" customWidth="1"/>
+    <col min="2" max="2" width="47.875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.25" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.75" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.25" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.75" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A2" s="59" t="s">
+    <row r="2" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-    </row>
-    <row r="3" spans="1:7" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+    </row>
+    <row r="3" spans="1:7" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="54"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="55"/>
+      <c r="C4" s="56"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
     </row>
-    <row r="5" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1693,23 +1693,23 @@
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
     </row>
-    <row r="6" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="56" t="s">
+    <row r="6" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="57" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>619</v>
+        <v>676</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
     </row>
-    <row r="7" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56"/>
+    <row r="7" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="57"/>
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
@@ -1721,21 +1721,21 @@
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
     </row>
-    <row r="8" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56"/>
+    <row r="8" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="57"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="8">
-        <v>619</v>
+        <v>676</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
     </row>
-    <row r="9" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="56" t="s">
+    <row r="9" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="57" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -1749,8 +1749,8 @@
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="56"/>
+    <row r="10" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="57"/>
       <c r="B10" s="3" t="s">
         <v>15</v>
       </c>
@@ -1762,8 +1762,8 @@
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
     </row>
-    <row r="11" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="56"/>
+    <row r="11" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="57"/>
       <c r="B11" s="3" t="s">
         <v>16</v>
       </c>
@@ -1775,8 +1775,8 @@
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
     </row>
-    <row r="12" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="56"/>
+    <row r="12" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="57"/>
       <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
@@ -1788,20 +1788,20 @@
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
     </row>
-    <row r="13" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="60" t="s">
         <v>18</v>
       </c>
       <c r="B13" s="60"/>
       <c r="C13" s="8">
-        <v>619</v>
+        <v>676</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -1810,7 +1810,7 @@
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
     </row>
-    <row r="15" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>0</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="44" t="s">
         <v>58</v>
       </c>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="G16" s="41"/>
     </row>
-    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45" t="s">
         <v>59</v>
       </c>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G17" s="41"/>
     </row>
-    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="45" t="s">
         <v>60</v>
       </c>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="G18" s="41"/>
     </row>
-    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="45" t="s">
         <v>61</v>
       </c>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="G19" s="41"/>
     </row>
-    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="45" t="s">
         <v>62</v>
       </c>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="G20" s="41"/>
     </row>
-    <row r="21" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="45" t="s">
         <v>63</v>
       </c>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="G21" s="43"/>
     </row>
-    <row r="22" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="45" t="s">
         <v>64</v>
       </c>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="G22" s="43"/>
     </row>
-    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="45" t="s">
         <v>65</v>
       </c>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="G23" s="43"/>
     </row>
-    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="45" t="s">
         <v>66</v>
       </c>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="G24" s="43"/>
     </row>
-    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="45" t="s">
         <v>67</v>
       </c>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G25" s="43"/>
     </row>
-    <row r="26" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
         <v>19</v>
       </c>
@@ -2062,8 +2062,8 @@
       <c r="F26" s="25"/>
       <c r="G26" s="26"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="56" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="57" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="12" t="s">
@@ -2072,17 +2072,17 @@
       <c r="C27" s="28">
         <v>2</v>
       </c>
-      <c r="D27" s="66" t="s">
+      <c r="D27" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="66" t="s">
+      <c r="E27" s="52" t="s">
         <v>56</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="56"/>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="57"/>
       <c r="B28" s="12" t="s">
         <v>23</v>
       </c>
@@ -2098,15 +2098,15 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="56"/>
+    <row r="29" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="57"/>
       <c r="B29" s="12" t="s">
         <v>24</v>
       </c>
       <c r="C29" s="28">
         <v>1</v>
       </c>
-      <c r="D29" s="66" t="s">
+      <c r="D29" s="52" t="s">
         <v>56</v>
       </c>
       <c r="E29" s="35" t="s">
@@ -2126,57 +2126,57 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A9:A12"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.94" bottom="0.41" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:G29"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
     <col min="2" max="2" width="50" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="10.77734375" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="17.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="10.75" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A2" s="59" t="s">
+    <row r="2" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-    </row>
-    <row r="3" spans="1:7" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+    </row>
+    <row r="3" spans="1:7" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="54"/>
       <c r="D3" s="16"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="55"/>
+      <c r="C4" s="56"/>
       <c r="D4" s="16"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
     </row>
-    <row r="5" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -2189,23 +2189,23 @@
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
     </row>
-    <row r="6" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="56" t="s">
+    <row r="6" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="57" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
     </row>
-    <row r="7" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56"/>
+    <row r="7" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="57"/>
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
@@ -2217,21 +2217,21 @@
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
     </row>
-    <row r="8" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56"/>
+    <row r="8" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="57"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="8">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
     </row>
-    <row r="9" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="56" t="s">
+    <row r="9" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="57" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -2245,8 +2245,8 @@
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="56"/>
+    <row r="10" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="57"/>
       <c r="B10" s="3" t="s">
         <v>15</v>
       </c>
@@ -2258,8 +2258,8 @@
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
     </row>
-    <row r="11" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="56"/>
+    <row r="11" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="57"/>
       <c r="B11" s="3" t="s">
         <v>16</v>
       </c>
@@ -2271,8 +2271,8 @@
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
     </row>
-    <row r="12" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="56"/>
+    <row r="12" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="57"/>
       <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
@@ -2284,20 +2284,20 @@
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
     </row>
-    <row r="13" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="60" t="s">
         <v>18</v>
       </c>
       <c r="B13" s="60"/>
       <c r="C13" s="8">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -2306,7 +2306,7 @@
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
     </row>
-    <row r="15" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>0</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="47" t="s">
         <v>77</v>
       </c>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="G16" s="39"/>
     </row>
-    <row r="17" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="s">
         <v>78</v>
       </c>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="G17" s="39"/>
     </row>
-    <row r="18" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="48" t="s">
         <v>79</v>
       </c>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="G18" s="39"/>
     </row>
-    <row r="19" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="s">
         <v>80</v>
       </c>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="G19" s="39"/>
     </row>
-    <row r="20" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="48" t="s">
         <v>81</v>
       </c>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="G20" s="39"/>
     </row>
-    <row r="21" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="48" t="s">
         <v>82</v>
       </c>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G21" s="28"/>
     </row>
-    <row r="22" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="48" t="s">
         <v>83</v>
       </c>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="G22" s="28"/>
     </row>
-    <row r="23" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="48" t="s">
         <v>38</v>
       </c>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G23" s="28"/>
     </row>
-    <row r="24" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="48" t="s">
         <v>84</v>
       </c>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="G24" s="28"/>
     </row>
-    <row r="25" spans="1:7" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="48" t="s">
         <v>85</v>
       </c>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="G25" s="28"/>
     </row>
-    <row r="26" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
         <v>19</v>
       </c>
@@ -2558,8 +2558,8 @@
       <c r="F26" s="50"/>
       <c r="G26" s="51"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="63" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="64" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="12" t="s">
@@ -2568,17 +2568,17 @@
       <c r="C27" s="28">
         <v>2</v>
       </c>
-      <c r="D27" s="66" t="s">
+      <c r="D27" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="66" t="s">
+      <c r="E27" s="52" t="s">
         <v>56</v>
       </c>
       <c r="F27" s="28"/>
       <c r="G27" s="28"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="64"/>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="65"/>
       <c r="B28" s="12" t="s">
         <v>23</v>
       </c>
@@ -2594,15 +2594,15 @@
       <c r="F28" s="28"/>
       <c r="G28" s="28"/>
     </row>
-    <row r="29" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="65"/>
+    <row r="29" spans="1:7" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="66"/>
       <c r="B29" s="12" t="s">
         <v>24</v>
       </c>
       <c r="C29" s="28">
         <v>1</v>
       </c>
-      <c r="D29" s="66" t="s">
+      <c r="D29" s="52" t="s">
         <v>56</v>
       </c>
       <c r="E29" s="35" t="s">
@@ -2622,7 +2622,7 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="B5:C5"/>
   </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0.97" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>